<commit_message>
🍏 Processed total 110 companies from 2025_Tier_1_BATCH_211-600 ( Found 624😱 New Contacts )+ titles to be removed Updated ⬆️ + 📝 DOCUMENTATION UPDATE ✅ : How to Use Scrapper Utility > Step 1.5 & Post-Credit Scenes
</commit_message>
<xml_diff>
--- a/OLD_OUTPUT/run_20jul2026/apollo_people_search_20jul2026_145716.xlsx
+++ b/OLD_OUTPUT/run_20jul2026/apollo_people_search_20jul2026_145716.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30305"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="184" documentId="11_D2FCAEFE017C9F6BBFA3D674305BDA16B64096AA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2613F1DD-258A-4503-B83F-437576B00AE9}"/>
+  <xr:revisionPtr revIDLastSave="202" documentId="11_D2FCAEFE017C9F6BBFA3D674305BDA16B64096AA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{496B9C4A-6C04-4457-999C-2C67A5F8EDF8}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Contacts" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16980" uniqueCount="2260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16987" uniqueCount="2266">
   <si>
     <t>apollo_person_id</t>
   </si>
@@ -5625,16 +5625,34 @@
     <t>Integration Product Director</t>
   </si>
   <si>
+    <t>Senior Technical Program Manager, Product &amp; Platform Engineering | Mergers &amp; Acquisitions</t>
+  </si>
+  <si>
     <t>VP Sales Engineering &amp; Enablement</t>
   </si>
   <si>
+    <t>Software Engineer (Product Developer)</t>
+  </si>
+  <si>
     <t>Vice President of Solution Engineering</t>
   </si>
   <si>
+    <t>Staff Product Engineer</t>
+  </si>
+  <si>
     <t>Director / Socio Fundador</t>
   </si>
   <si>
+    <t>Staff AI Scientist – AI Product Engineering</t>
+  </si>
+  <si>
+    <t>Product Engineering</t>
+  </si>
+  <si>
     <t>Chief Operating Officer / Head of Sales / Executive Director</t>
+  </si>
+  <si>
+    <t>Product Engineering Intern – Crash &amp; Safety</t>
   </si>
   <si>
     <t>BDM // Empowering the Long-tail of the Road Freight Industry Through Technology // Co Founder</t>
@@ -6820,7 +6838,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -6840,6 +6858,14 @@
       <color rgb="FF000000"/>
       <name val="-Apple-System"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -6862,7 +6888,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -6870,6 +6896,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -59054,10 +59081,11 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73124581-F44C-485A-95D5-2C8203FF0E02}">
-  <dimension ref="A1:A608"/>
+  <dimension ref="A1:H608"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="65" customWidth="1"/>
+    <col min="8" max="8" width="82.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="16.5">
@@ -59220,204 +59248,225 @@
         <v>1845</v>
       </c>
     </row>
-    <row r="33" spans="1:1" ht="16.5">
+    <row r="33" spans="1:8" ht="16.5">
       <c r="A33" s="2" t="s">
         <v>1846</v>
       </c>
     </row>
-    <row r="34" spans="1:1" ht="16.5">
+    <row r="34" spans="1:8" ht="16.5">
       <c r="A34" s="2" t="s">
         <v>1417</v>
       </c>
     </row>
-    <row r="35" spans="1:1" ht="16.5">
+    <row r="35" spans="1:8" ht="16.5">
       <c r="A35" s="2" t="s">
         <v>1847</v>
       </c>
     </row>
-    <row r="36" spans="1:1" ht="16.5">
+    <row r="36" spans="1:8" ht="16.5">
       <c r="A36" s="2" t="s">
         <v>1848</v>
       </c>
     </row>
-    <row r="37" spans="1:1" ht="16.5">
+    <row r="37" spans="1:8" ht="16.5">
       <c r="A37" s="2" t="s">
         <v>1849</v>
       </c>
     </row>
-    <row r="38" spans="1:1" ht="16.5">
+    <row r="38" spans="1:8" ht="16.5">
       <c r="A38" s="2" t="s">
         <v>1850</v>
       </c>
     </row>
-    <row r="39" spans="1:1" ht="16.5">
+    <row r="39" spans="1:8" ht="16.5">
       <c r="A39" s="2" t="s">
         <v>1851</v>
       </c>
     </row>
-    <row r="40" spans="1:1" ht="16.5">
+    <row r="40" spans="1:8" ht="16.5">
       <c r="A40" s="2" t="s">
         <v>1852</v>
       </c>
     </row>
-    <row r="41" spans="1:1" ht="16.5">
+    <row r="41" spans="1:8" ht="16.5">
       <c r="A41" s="2" t="s">
         <v>1853</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" ht="16.5">
+      <c r="H41" s="3" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="16.5">
       <c r="A42" s="2" t="s">
         <v>1854</v>
       </c>
     </row>
-    <row r="43" spans="1:1" ht="16.5">
+    <row r="43" spans="1:8" ht="16.5">
       <c r="A43" s="2" t="s">
         <v>1855</v>
       </c>
     </row>
-    <row r="44" spans="1:1" ht="16.5">
+    <row r="44" spans="1:8" ht="16.5">
       <c r="A44" s="2" t="s">
         <v>1856</v>
       </c>
     </row>
-    <row r="45" spans="1:1" ht="16.5">
+    <row r="45" spans="1:8" ht="16.5">
       <c r="A45" s="2" t="s">
         <v>1857</v>
       </c>
     </row>
-    <row r="46" spans="1:1" ht="33.75">
+    <row r="46" spans="1:8" ht="16.5">
       <c r="A46" s="2" t="s">
         <v>1858</v>
       </c>
     </row>
-    <row r="47" spans="1:1" ht="16.5">
+    <row r="47" spans="1:8" ht="16.5">
       <c r="A47" s="2" t="s">
         <v>1859</v>
       </c>
     </row>
-    <row r="48" spans="1:1" ht="16.5">
+    <row r="48" spans="1:8" ht="16.5">
       <c r="A48" s="2" t="s">
         <v>1559</v>
       </c>
     </row>
-    <row r="49" spans="1:1" ht="16.5">
+    <row r="49" spans="1:8" ht="16.5">
       <c r="A49" s="2" t="s">
         <v>1860</v>
       </c>
     </row>
-    <row r="50" spans="1:1" ht="16.5">
+    <row r="50" spans="1:8" ht="16.5">
       <c r="A50" s="2" t="s">
         <v>1861</v>
       </c>
     </row>
-    <row r="51" spans="1:1" ht="16.5">
+    <row r="51" spans="1:8" ht="16.5">
       <c r="A51" s="2" t="s">
         <v>1862</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" ht="16.5">
+      <c r="H51" t="s">
+        <v>1863</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" ht="16.5">
       <c r="A52" s="2" t="s">
-        <v>1863</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" ht="16.5">
+        <v>1864</v>
+      </c>
+      <c r="H52" t="s">
+        <v>1865</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" ht="16.5">
       <c r="A53" s="2" t="s">
-        <v>1864</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1" ht="16.5">
+        <v>1866</v>
+      </c>
+      <c r="H53" t="s">
+        <v>1867</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" ht="16.5">
       <c r="A54" s="2" t="s">
-        <v>1865</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" ht="33.75">
+        <v>1868</v>
+      </c>
+      <c r="H54" t="s">
+        <v>1869</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" ht="16.5">
       <c r="A55" s="2" t="s">
         <v>1721</v>
       </c>
-    </row>
-    <row r="56" spans="1:1" ht="33.75">
+      <c r="H55" t="s">
+        <v>1870</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" ht="16.5">
       <c r="A56" s="2" t="s">
-        <v>1866</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" ht="50.25">
+        <v>1871</v>
+      </c>
+      <c r="H56" t="s">
+        <v>1872</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" ht="33.75">
       <c r="A57" s="2" t="s">
-        <v>1867</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1" ht="33.75">
+        <v>1873</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" ht="16.5">
       <c r="A58" s="2" t="s">
-        <v>1868</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" ht="33.75">
+        <v>1874</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" ht="16.5">
       <c r="A59" s="2" t="s">
-        <v>1869</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1" ht="16.5">
+        <v>1875</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" ht="16.5">
       <c r="A60" s="2" t="s">
-        <v>1870</v>
-      </c>
-    </row>
-    <row r="61" spans="1:1" ht="16.5">
+        <v>1876</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" ht="16.5">
       <c r="A61" s="2" t="s">
         <v>1472</v>
       </c>
     </row>
-    <row r="62" spans="1:1" ht="33.75">
+    <row r="62" spans="1:8" ht="16.5">
       <c r="A62" s="2" t="s">
-        <v>1871</v>
-      </c>
-    </row>
-    <row r="63" spans="1:1" ht="16.5">
+        <v>1877</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" ht="16.5">
       <c r="A63" s="2" t="s">
         <v>1428</v>
       </c>
     </row>
-    <row r="64" spans="1:1" ht="16.5">
+    <row r="64" spans="1:8" ht="16.5">
       <c r="A64" s="2" t="s">
-        <v>1872</v>
+        <v>1878</v>
       </c>
     </row>
     <row r="65" spans="1:1" ht="16.5">
       <c r="A65" s="2" t="s">
-        <v>1873</v>
+        <v>1879</v>
       </c>
     </row>
     <row r="66" spans="1:1" ht="16.5">
       <c r="A66" s="2" t="s">
-        <v>1874</v>
+        <v>1880</v>
       </c>
     </row>
     <row r="67" spans="1:1" ht="16.5">
       <c r="A67" s="2" t="s">
-        <v>1875</v>
+        <v>1881</v>
       </c>
     </row>
     <row r="68" spans="1:1" ht="16.5">
       <c r="A68" s="2" t="s">
-        <v>1876</v>
+        <v>1882</v>
       </c>
     </row>
     <row r="69" spans="1:1" ht="16.5">
       <c r="A69" s="2" t="s">
-        <v>1877</v>
+        <v>1883</v>
       </c>
     </row>
     <row r="70" spans="1:1" ht="33.75">
       <c r="A70" s="2" t="s">
-        <v>1878</v>
+        <v>1884</v>
       </c>
     </row>
     <row r="71" spans="1:1" ht="16.5">
       <c r="A71" s="2" t="s">
-        <v>1879</v>
-      </c>
-    </row>
-    <row r="72" spans="1:1" ht="33.75">
+        <v>1885</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" ht="16.5">
       <c r="A72" s="2" t="s">
-        <v>1880</v>
+        <v>1886</v>
       </c>
     </row>
     <row r="73" spans="1:1" ht="16.5">
@@ -59425,19 +59474,19 @@
         <v>1460</v>
       </c>
     </row>
-    <row r="74" spans="1:1" ht="33.75">
+    <row r="74" spans="1:1" ht="16.5">
       <c r="A74" s="2" t="s">
-        <v>1881</v>
+        <v>1887</v>
       </c>
     </row>
     <row r="75" spans="1:1" ht="16.5">
       <c r="A75" s="2" t="s">
-        <v>1882</v>
-      </c>
-    </row>
-    <row r="76" spans="1:1" ht="33.75">
+        <v>1888</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" ht="16.5">
       <c r="A76" s="2" t="s">
-        <v>1883</v>
+        <v>1889</v>
       </c>
     </row>
     <row r="77" spans="1:1" ht="16.5">
@@ -59447,142 +59496,142 @@
     </row>
     <row r="78" spans="1:1" ht="16.5">
       <c r="A78" s="2" t="s">
-        <v>1884</v>
+        <v>1890</v>
       </c>
     </row>
     <row r="79" spans="1:1" ht="16.5">
       <c r="A79" s="2" t="s">
-        <v>1885</v>
+        <v>1891</v>
       </c>
     </row>
     <row r="80" spans="1:1" ht="16.5">
       <c r="A80" s="2" t="s">
-        <v>1886</v>
+        <v>1892</v>
       </c>
     </row>
     <row r="81" spans="1:1" ht="16.5">
       <c r="A81" s="2" t="s">
-        <v>1887</v>
+        <v>1893</v>
       </c>
     </row>
     <row r="82" spans="1:1" ht="16.5">
       <c r="A82" s="2" t="s">
-        <v>1888</v>
+        <v>1894</v>
       </c>
     </row>
     <row r="83" spans="1:1" ht="16.5">
       <c r="A83" s="2" t="s">
-        <v>1889</v>
-      </c>
-    </row>
-    <row r="84" spans="1:1" ht="33.75">
+        <v>1895</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" ht="16.5">
       <c r="A84" s="2" t="s">
-        <v>1890</v>
+        <v>1896</v>
       </c>
     </row>
     <row r="85" spans="1:1" ht="16.5">
       <c r="A85" s="2" t="s">
-        <v>1891</v>
+        <v>1897</v>
       </c>
     </row>
     <row r="86" spans="1:1" ht="16.5">
       <c r="A86" s="2" t="s">
-        <v>1892</v>
+        <v>1898</v>
       </c>
     </row>
     <row r="87" spans="1:1" ht="16.5">
       <c r="A87" s="2" t="s">
-        <v>1893</v>
+        <v>1899</v>
       </c>
     </row>
     <row r="88" spans="1:1" ht="16.5">
       <c r="A88" s="2" t="s">
-        <v>1894</v>
-      </c>
-    </row>
-    <row r="89" spans="1:1" ht="33.75">
+        <v>1900</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" ht="16.5">
       <c r="A89" s="2" t="s">
-        <v>1895</v>
+        <v>1901</v>
       </c>
     </row>
     <row r="90" spans="1:1" ht="16.5">
       <c r="A90" s="2" t="s">
-        <v>1896</v>
+        <v>1902</v>
       </c>
     </row>
     <row r="91" spans="1:1" ht="16.5">
       <c r="A91" s="2" t="s">
-        <v>1897</v>
+        <v>1903</v>
       </c>
     </row>
     <row r="92" spans="1:1" ht="16.5">
       <c r="A92" s="2" t="s">
-        <v>1898</v>
+        <v>1904</v>
       </c>
     </row>
     <row r="93" spans="1:1" ht="16.5">
       <c r="A93" s="2" t="s">
-        <v>1899</v>
-      </c>
-    </row>
-    <row r="94" spans="1:1" ht="33.75">
+        <v>1905</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" ht="16.5">
       <c r="A94" s="2" t="s">
-        <v>1900</v>
+        <v>1906</v>
       </c>
     </row>
     <row r="95" spans="1:1" ht="16.5">
       <c r="A95" s="2" t="s">
-        <v>1901</v>
+        <v>1907</v>
       </c>
     </row>
     <row r="96" spans="1:1" ht="16.5">
       <c r="A96" s="2" t="s">
-        <v>1902</v>
+        <v>1908</v>
       </c>
     </row>
     <row r="97" spans="1:1" ht="16.5">
       <c r="A97" s="2" t="s">
-        <v>1903</v>
+        <v>1909</v>
       </c>
     </row>
     <row r="98" spans="1:1" ht="16.5">
       <c r="A98" s="2" t="s">
-        <v>1904</v>
-      </c>
-    </row>
-    <row r="99" spans="1:1" ht="33.75">
+        <v>1910</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" ht="16.5">
       <c r="A99" s="2" t="s">
-        <v>1905</v>
-      </c>
-    </row>
-    <row r="100" spans="1:1" ht="33.75">
+        <v>1911</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" ht="16.5">
       <c r="A100" s="2" t="s">
-        <v>1906</v>
+        <v>1912</v>
       </c>
     </row>
     <row r="101" spans="1:1" ht="16.5">
       <c r="A101" s="2" t="s">
-        <v>1907</v>
+        <v>1913</v>
       </c>
     </row>
     <row r="102" spans="1:1" ht="16.5">
       <c r="A102" s="2" t="s">
-        <v>1908</v>
+        <v>1914</v>
       </c>
     </row>
     <row r="103" spans="1:1" ht="16.5">
       <c r="A103" s="2" t="s">
-        <v>1909</v>
+        <v>1915</v>
       </c>
     </row>
     <row r="104" spans="1:1" ht="16.5">
       <c r="A104" s="2" t="s">
-        <v>1910</v>
+        <v>1916</v>
       </c>
     </row>
     <row r="105" spans="1:1" ht="33.75">
       <c r="A105" s="2" t="s">
-        <v>1911</v>
+        <v>1917</v>
       </c>
     </row>
     <row r="106" spans="1:1" ht="16.5">
@@ -59592,12 +59641,12 @@
     </row>
     <row r="107" spans="1:1" ht="16.5">
       <c r="A107" s="2" t="s">
-        <v>1912</v>
+        <v>1918</v>
       </c>
     </row>
     <row r="108" spans="1:1" ht="16.5">
       <c r="A108" s="2" t="s">
-        <v>1913</v>
+        <v>1919</v>
       </c>
     </row>
     <row r="109" spans="1:1" ht="16.5">
@@ -59607,77 +59656,77 @@
     </row>
     <row r="110" spans="1:1" ht="16.5">
       <c r="A110" s="2" t="s">
-        <v>1914</v>
+        <v>1920</v>
       </c>
     </row>
     <row r="111" spans="1:1" ht="16.5">
       <c r="A111" s="2" t="s">
-        <v>1915</v>
+        <v>1921</v>
       </c>
     </row>
     <row r="112" spans="1:1" ht="16.5">
       <c r="A112" s="2" t="s">
-        <v>1916</v>
-      </c>
-    </row>
-    <row r="113" spans="1:1" ht="33.75">
+        <v>1922</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" ht="16.5">
       <c r="A113" s="2" t="s">
-        <v>1917</v>
+        <v>1923</v>
       </c>
     </row>
     <row r="114" spans="1:1" ht="16.5">
       <c r="A114" s="2" t="s">
-        <v>1918</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="115" spans="1:1" ht="16.5">
       <c r="A115" s="2" t="s">
-        <v>1919</v>
+        <v>1925</v>
       </c>
     </row>
     <row r="116" spans="1:1" ht="16.5">
       <c r="A116" s="2" t="s">
-        <v>1920</v>
+        <v>1926</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="16.5">
       <c r="A117" s="2" t="s">
-        <v>1921</v>
+        <v>1927</v>
       </c>
     </row>
     <row r="118" spans="1:1" ht="16.5">
       <c r="A118" s="2" t="s">
-        <v>1922</v>
+        <v>1928</v>
       </c>
     </row>
     <row r="119" spans="1:1" ht="16.5">
       <c r="A119" s="2" t="s">
-        <v>1923</v>
+        <v>1929</v>
       </c>
     </row>
     <row r="120" spans="1:1" ht="33.75">
       <c r="A120" s="2" t="s">
-        <v>1924</v>
+        <v>1930</v>
       </c>
     </row>
     <row r="121" spans="1:1" ht="16.5">
       <c r="A121" s="2" t="s">
-        <v>1925</v>
+        <v>1931</v>
       </c>
     </row>
     <row r="122" spans="1:1" ht="16.5">
       <c r="A122" s="2" t="s">
-        <v>1926</v>
+        <v>1932</v>
       </c>
     </row>
     <row r="123" spans="1:1" ht="16.5">
       <c r="A123" s="2" t="s">
-        <v>1927</v>
+        <v>1933</v>
       </c>
     </row>
     <row r="124" spans="1:1" ht="16.5">
       <c r="A124" s="2" t="s">
-        <v>1928</v>
+        <v>1934</v>
       </c>
     </row>
     <row r="125" spans="1:1" ht="16.5">
@@ -59687,42 +59736,42 @@
     </row>
     <row r="126" spans="1:1" ht="16.5">
       <c r="A126" s="2" t="s">
-        <v>1929</v>
+        <v>1935</v>
       </c>
     </row>
     <row r="127" spans="1:1" ht="16.5">
       <c r="A127" s="2" t="s">
-        <v>1930</v>
+        <v>1936</v>
       </c>
     </row>
     <row r="128" spans="1:1" ht="16.5">
       <c r="A128" s="2" t="s">
-        <v>1931</v>
+        <v>1937</v>
       </c>
     </row>
     <row r="129" spans="1:1" ht="33.75">
       <c r="A129" s="2" t="s">
-        <v>1932</v>
+        <v>1938</v>
       </c>
     </row>
     <row r="130" spans="1:1" ht="16.5">
       <c r="A130" s="2" t="s">
-        <v>1933</v>
+        <v>1939</v>
       </c>
     </row>
     <row r="131" spans="1:1" ht="16.5">
       <c r="A131" s="2" t="s">
-        <v>1934</v>
+        <v>1940</v>
       </c>
     </row>
     <row r="132" spans="1:1" ht="16.5">
       <c r="A132" s="2" t="s">
-        <v>1935</v>
+        <v>1941</v>
       </c>
     </row>
     <row r="133" spans="1:1" ht="33.75">
       <c r="A133" s="2" t="s">
-        <v>1936</v>
+        <v>1942</v>
       </c>
     </row>
     <row r="134" spans="1:1" ht="16.5">
@@ -59732,57 +59781,57 @@
     </row>
     <row r="135" spans="1:1" ht="16.5">
       <c r="A135" s="2" t="s">
-        <v>1937</v>
+        <v>1943</v>
       </c>
     </row>
     <row r="136" spans="1:1" ht="16.5">
       <c r="A136" s="2" t="s">
-        <v>1938</v>
+        <v>1944</v>
       </c>
     </row>
     <row r="137" spans="1:1" ht="16.5">
       <c r="A137" s="2" t="s">
-        <v>1939</v>
+        <v>1945</v>
       </c>
     </row>
     <row r="138" spans="1:1" ht="16.5">
       <c r="A138" s="2" t="s">
-        <v>1940</v>
+        <v>1946</v>
       </c>
     </row>
     <row r="139" spans="1:1" ht="33.75">
       <c r="A139" s="2" t="s">
-        <v>1941</v>
+        <v>1947</v>
       </c>
     </row>
     <row r="140" spans="1:1" ht="33.75">
       <c r="A140" s="2" t="s">
-        <v>1942</v>
+        <v>1948</v>
       </c>
     </row>
     <row r="141" spans="1:1" ht="16.5">
       <c r="A141" s="2" t="s">
-        <v>1943</v>
+        <v>1949</v>
       </c>
     </row>
     <row r="142" spans="1:1" ht="16.5">
       <c r="A142" s="2" t="s">
-        <v>1944</v>
+        <v>1950</v>
       </c>
     </row>
     <row r="143" spans="1:1" ht="16.5">
       <c r="A143" s="2" t="s">
-        <v>1945</v>
+        <v>1951</v>
       </c>
     </row>
     <row r="144" spans="1:1" ht="16.5">
       <c r="A144" s="2" t="s">
-        <v>1946</v>
+        <v>1952</v>
       </c>
     </row>
     <row r="145" spans="1:1" ht="16.5">
       <c r="A145" s="2" t="s">
-        <v>1947</v>
+        <v>1953</v>
       </c>
     </row>
     <row r="146" spans="1:1" ht="16.5">
@@ -59792,57 +59841,57 @@
     </row>
     <row r="147" spans="1:1" ht="16.5">
       <c r="A147" s="2" t="s">
-        <v>1948</v>
+        <v>1954</v>
       </c>
     </row>
     <row r="148" spans="1:1" ht="33.75">
       <c r="A148" s="2" t="s">
-        <v>1949</v>
+        <v>1955</v>
       </c>
     </row>
     <row r="149" spans="1:1" ht="33.75">
       <c r="A149" s="2" t="s">
-        <v>1950</v>
+        <v>1956</v>
       </c>
     </row>
     <row r="150" spans="1:1" ht="33.75">
       <c r="A150" s="2" t="s">
-        <v>1951</v>
+        <v>1957</v>
       </c>
     </row>
     <row r="151" spans="1:1" ht="16.5">
       <c r="A151" s="2" t="s">
-        <v>1952</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="152" spans="1:1" ht="33.75">
       <c r="A152" s="2" t="s">
-        <v>1953</v>
+        <v>1959</v>
       </c>
     </row>
     <row r="153" spans="1:1" ht="16.5">
       <c r="A153" s="2" t="s">
-        <v>1954</v>
+        <v>1960</v>
       </c>
     </row>
     <row r="154" spans="1:1" ht="16.5">
       <c r="A154" s="2" t="s">
-        <v>1955</v>
+        <v>1961</v>
       </c>
     </row>
     <row r="155" spans="1:1" ht="16.5">
       <c r="A155" s="2" t="s">
-        <v>1956</v>
+        <v>1962</v>
       </c>
     </row>
     <row r="156" spans="1:1" ht="16.5">
       <c r="A156" s="2" t="s">
-        <v>1957</v>
+        <v>1963</v>
       </c>
     </row>
     <row r="157" spans="1:1" ht="16.5">
       <c r="A157" s="2" t="s">
-        <v>1958</v>
+        <v>1964</v>
       </c>
     </row>
     <row r="158" spans="1:1" ht="16.5">
@@ -59852,27 +59901,27 @@
     </row>
     <row r="159" spans="1:1" ht="16.5">
       <c r="A159" s="2" t="s">
-        <v>1959</v>
+        <v>1965</v>
       </c>
     </row>
     <row r="160" spans="1:1" ht="16.5">
       <c r="A160" s="2" t="s">
-        <v>1960</v>
+        <v>1966</v>
       </c>
     </row>
     <row r="161" spans="1:1" ht="16.5">
       <c r="A161" s="2" t="s">
-        <v>1961</v>
+        <v>1967</v>
       </c>
     </row>
     <row r="162" spans="1:1" ht="33.75">
       <c r="A162" s="2" t="s">
-        <v>1962</v>
+        <v>1968</v>
       </c>
     </row>
     <row r="163" spans="1:1" ht="33.75">
       <c r="A163" s="2" t="s">
-        <v>1963</v>
+        <v>1969</v>
       </c>
     </row>
     <row r="164" spans="1:1" ht="16.5">
@@ -59882,52 +59931,52 @@
     </row>
     <row r="165" spans="1:1" ht="16.5">
       <c r="A165" s="2" t="s">
-        <v>1964</v>
+        <v>1970</v>
       </c>
     </row>
     <row r="166" spans="1:1" ht="33.75">
       <c r="A166" s="2" t="s">
-        <v>1965</v>
+        <v>1971</v>
       </c>
     </row>
     <row r="167" spans="1:1" ht="16.5">
       <c r="A167" s="2" t="s">
-        <v>1966</v>
+        <v>1972</v>
       </c>
     </row>
     <row r="168" spans="1:1" ht="16.5">
       <c r="A168" s="2" t="s">
-        <v>1967</v>
+        <v>1973</v>
       </c>
     </row>
     <row r="169" spans="1:1" ht="16.5">
       <c r="A169" s="2" t="s">
-        <v>1968</v>
+        <v>1974</v>
       </c>
     </row>
     <row r="170" spans="1:1" ht="33.75">
       <c r="A170" s="2" t="s">
-        <v>1969</v>
+        <v>1975</v>
       </c>
     </row>
     <row r="171" spans="1:1" ht="33.75">
       <c r="A171" s="2" t="s">
-        <v>1970</v>
+        <v>1976</v>
       </c>
     </row>
     <row r="172" spans="1:1" ht="66.75">
       <c r="A172" s="2" t="s">
-        <v>1971</v>
+        <v>1977</v>
       </c>
     </row>
     <row r="173" spans="1:1" ht="16.5">
       <c r="A173" s="2" t="s">
-        <v>1972</v>
+        <v>1978</v>
       </c>
     </row>
     <row r="174" spans="1:1" ht="33.75">
       <c r="A174" s="2" t="s">
-        <v>1973</v>
+        <v>1979</v>
       </c>
     </row>
     <row r="175" spans="1:1" ht="16.5">
@@ -59937,172 +59986,172 @@
     </row>
     <row r="176" spans="1:1" ht="33.75">
       <c r="A176" s="2" t="s">
-        <v>1974</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="177" spans="1:1" ht="16.5">
       <c r="A177" s="2" t="s">
-        <v>1975</v>
+        <v>1981</v>
       </c>
     </row>
     <row r="178" spans="1:1" ht="16.5">
       <c r="A178" s="2" t="s">
-        <v>1976</v>
+        <v>1982</v>
       </c>
     </row>
     <row r="179" spans="1:1" ht="16.5">
       <c r="A179" s="2" t="s">
-        <v>1977</v>
+        <v>1983</v>
       </c>
     </row>
     <row r="180" spans="1:1" ht="16.5">
       <c r="A180" s="2" t="s">
-        <v>1978</v>
+        <v>1984</v>
       </c>
     </row>
     <row r="181" spans="1:1" ht="16.5">
       <c r="A181" s="2" t="s">
-        <v>1979</v>
+        <v>1985</v>
       </c>
     </row>
     <row r="182" spans="1:1" ht="16.5">
       <c r="A182" s="2" t="s">
-        <v>1980</v>
+        <v>1986</v>
       </c>
     </row>
     <row r="183" spans="1:1" ht="16.5">
       <c r="A183" s="2" t="s">
-        <v>1981</v>
+        <v>1987</v>
       </c>
     </row>
     <row r="184" spans="1:1" ht="33.75">
       <c r="A184" s="2" t="s">
-        <v>1982</v>
+        <v>1988</v>
       </c>
     </row>
     <row r="185" spans="1:1" ht="16.5">
       <c r="A185" s="2" t="s">
-        <v>1983</v>
+        <v>1989</v>
       </c>
     </row>
     <row r="186" spans="1:1" ht="16.5">
       <c r="A186" s="2" t="s">
-        <v>1984</v>
+        <v>1990</v>
       </c>
     </row>
     <row r="187" spans="1:1" ht="16.5">
       <c r="A187" s="2" t="s">
-        <v>1985</v>
+        <v>1991</v>
       </c>
     </row>
     <row r="188" spans="1:1" ht="16.5">
       <c r="A188" s="2" t="s">
-        <v>1986</v>
+        <v>1992</v>
       </c>
     </row>
     <row r="189" spans="1:1" ht="33.75">
       <c r="A189" s="2" t="s">
-        <v>1987</v>
+        <v>1993</v>
       </c>
     </row>
     <row r="190" spans="1:1" ht="16.5">
       <c r="A190" s="2" t="s">
-        <v>1988</v>
+        <v>1994</v>
       </c>
     </row>
     <row r="191" spans="1:1" ht="16.5">
       <c r="A191" s="2" t="s">
-        <v>1989</v>
+        <v>1995</v>
       </c>
     </row>
     <row r="192" spans="1:1" ht="16.5">
       <c r="A192" s="2" t="s">
-        <v>1990</v>
+        <v>1996</v>
       </c>
     </row>
     <row r="193" spans="1:1" ht="33.75">
       <c r="A193" s="2" t="s">
-        <v>1991</v>
+        <v>1997</v>
       </c>
     </row>
     <row r="194" spans="1:1" ht="33.75">
       <c r="A194" s="2" t="s">
-        <v>1992</v>
+        <v>1998</v>
       </c>
     </row>
     <row r="195" spans="1:1" ht="16.5">
       <c r="A195" s="2" t="s">
-        <v>1993</v>
+        <v>1999</v>
       </c>
     </row>
     <row r="196" spans="1:1" ht="33.75">
       <c r="A196" s="2" t="s">
-        <v>1994</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="197" spans="1:1" ht="33.75">
       <c r="A197" s="2" t="s">
-        <v>1995</v>
+        <v>2001</v>
       </c>
     </row>
     <row r="198" spans="1:1" ht="16.5">
       <c r="A198" s="2" t="s">
-        <v>1996</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="199" spans="1:1" ht="33.75">
       <c r="A199" s="2" t="s">
-        <v>1997</v>
+        <v>2003</v>
       </c>
     </row>
     <row r="200" spans="1:1" ht="16.5">
       <c r="A200" s="2" t="s">
-        <v>1998</v>
+        <v>2004</v>
       </c>
     </row>
     <row r="201" spans="1:1" ht="16.5">
       <c r="A201" s="2" t="s">
-        <v>1999</v>
+        <v>2005</v>
       </c>
     </row>
     <row r="202" spans="1:1" ht="50.25">
       <c r="A202" s="2" t="s">
-        <v>2000</v>
+        <v>2006</v>
       </c>
     </row>
     <row r="203" spans="1:1" ht="16.5">
       <c r="A203" s="2" t="s">
-        <v>2001</v>
+        <v>2007</v>
       </c>
     </row>
     <row r="204" spans="1:1" ht="16.5">
       <c r="A204" s="2" t="s">
-        <v>2002</v>
+        <v>2008</v>
       </c>
     </row>
     <row r="205" spans="1:1" ht="16.5">
       <c r="A205" s="2" t="s">
-        <v>2003</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="206" spans="1:1" ht="16.5">
       <c r="A206" s="2" t="s">
-        <v>2004</v>
+        <v>2010</v>
       </c>
     </row>
     <row r="207" spans="1:1" ht="16.5">
       <c r="A207" s="2" t="s">
-        <v>2005</v>
+        <v>2011</v>
       </c>
     </row>
     <row r="208" spans="1:1" ht="33.75">
       <c r="A208" s="2" t="s">
-        <v>2006</v>
+        <v>2012</v>
       </c>
     </row>
     <row r="209" spans="1:1" ht="16.5">
       <c r="A209" s="2" t="s">
-        <v>2007</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="210" spans="1:1" ht="16.5">
@@ -60112,12 +60161,12 @@
     </row>
     <row r="211" spans="1:1" ht="33.75">
       <c r="A211" s="2" t="s">
-        <v>2008</v>
+        <v>2014</v>
       </c>
     </row>
     <row r="212" spans="1:1" ht="16.5">
       <c r="A212" s="2" t="s">
-        <v>2009</v>
+        <v>2015</v>
       </c>
     </row>
     <row r="213" spans="1:1" ht="33.75">
@@ -60127,62 +60176,62 @@
     </row>
     <row r="214" spans="1:1" ht="16.5">
       <c r="A214" s="2" t="s">
-        <v>2010</v>
+        <v>2016</v>
       </c>
     </row>
     <row r="215" spans="1:1" ht="16.5">
       <c r="A215" s="2" t="s">
-        <v>2011</v>
+        <v>2017</v>
       </c>
     </row>
     <row r="216" spans="1:1" ht="16.5">
       <c r="A216" s="2" t="s">
-        <v>2012</v>
+        <v>2018</v>
       </c>
     </row>
     <row r="217" spans="1:1" ht="16.5">
       <c r="A217" s="2" t="s">
-        <v>2013</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="218" spans="1:1" ht="66.75">
       <c r="A218" s="2" t="s">
-        <v>2014</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="219" spans="1:1" ht="16.5">
       <c r="A219" s="2" t="s">
-        <v>2015</v>
+        <v>2021</v>
       </c>
     </row>
     <row r="220" spans="1:1" ht="16.5">
       <c r="A220" s="2" t="s">
-        <v>2016</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="221" spans="1:1" ht="33.75">
       <c r="A221" s="2" t="s">
-        <v>2017</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="222" spans="1:1" ht="16.5">
       <c r="A222" s="2" t="s">
-        <v>2018</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="223" spans="1:1" ht="16.5">
       <c r="A223" s="2" t="s">
-        <v>2019</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="224" spans="1:1" ht="33.75">
       <c r="A224" s="2" t="s">
-        <v>2020</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="225" spans="1:1" ht="16.5">
       <c r="A225" s="2" t="s">
-        <v>2021</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="226" spans="1:1" ht="16.5">
@@ -60192,37 +60241,37 @@
     </row>
     <row r="227" spans="1:1" ht="16.5">
       <c r="A227" s="2" t="s">
-        <v>2022</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="228" spans="1:1" ht="16.5">
       <c r="A228" s="2" t="s">
-        <v>2023</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="229" spans="1:1" ht="16.5">
       <c r="A229" s="2" t="s">
-        <v>1893</v>
+        <v>1899</v>
       </c>
     </row>
     <row r="230" spans="1:1" ht="16.5">
       <c r="A230" s="2" t="s">
-        <v>2024</v>
+        <v>2030</v>
       </c>
     </row>
     <row r="231" spans="1:1" ht="33.75">
       <c r="A231" s="2" t="s">
-        <v>2025</v>
+        <v>2031</v>
       </c>
     </row>
     <row r="232" spans="1:1" ht="16.5">
       <c r="A232" s="2" t="s">
-        <v>2026</v>
+        <v>2032</v>
       </c>
     </row>
     <row r="233" spans="1:1" ht="33.75">
       <c r="A233" s="2" t="s">
-        <v>2027</v>
+        <v>2033</v>
       </c>
     </row>
     <row r="234" spans="1:1" ht="16.5">
@@ -60232,82 +60281,82 @@
     </row>
     <row r="235" spans="1:1" ht="16.5">
       <c r="A235" s="2" t="s">
-        <v>2028</v>
+        <v>2034</v>
       </c>
     </row>
     <row r="236" spans="1:1" ht="16.5">
       <c r="A236" s="2" t="s">
-        <v>2029</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="237" spans="1:1" ht="16.5">
       <c r="A237" s="2" t="s">
-        <v>2030</v>
+        <v>2036</v>
       </c>
     </row>
     <row r="238" spans="1:1" ht="16.5">
       <c r="A238" s="2" t="s">
-        <v>2031</v>
+        <v>2037</v>
       </c>
     </row>
     <row r="239" spans="1:1" ht="16.5">
       <c r="A239" s="2" t="s">
-        <v>2032</v>
+        <v>2038</v>
       </c>
     </row>
     <row r="240" spans="1:1" ht="16.5">
       <c r="A240" s="2" t="s">
-        <v>2033</v>
+        <v>2039</v>
       </c>
     </row>
     <row r="241" spans="1:1" ht="16.5">
       <c r="A241" s="2" t="s">
-        <v>2034</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="242" spans="1:1" ht="16.5">
       <c r="A242" s="2" t="s">
-        <v>2035</v>
+        <v>2041</v>
       </c>
     </row>
     <row r="243" spans="1:1" ht="16.5">
       <c r="A243" s="2" t="s">
-        <v>2036</v>
+        <v>2042</v>
       </c>
     </row>
     <row r="244" spans="1:1" ht="33.75">
       <c r="A244" s="2" t="s">
-        <v>2037</v>
+        <v>2043</v>
       </c>
     </row>
     <row r="245" spans="1:1" ht="16.5">
       <c r="A245" s="2" t="s">
-        <v>2038</v>
+        <v>2044</v>
       </c>
     </row>
     <row r="246" spans="1:1" ht="33.75">
       <c r="A246" s="2" t="s">
-        <v>2039</v>
+        <v>2045</v>
       </c>
     </row>
     <row r="247" spans="1:1" ht="16.5">
       <c r="A247" s="2" t="s">
-        <v>2040</v>
+        <v>2046</v>
       </c>
     </row>
     <row r="248" spans="1:1" ht="16.5">
       <c r="A248" s="2" t="s">
-        <v>2041</v>
+        <v>2047</v>
       </c>
     </row>
     <row r="249" spans="1:1" ht="16.5">
       <c r="A249" s="2" t="s">
-        <v>2042</v>
+        <v>2048</v>
       </c>
     </row>
     <row r="250" spans="1:1" ht="16.5">
       <c r="A250" s="2" t="s">
-        <v>2043</v>
+        <v>2049</v>
       </c>
     </row>
     <row r="251" spans="1:1" ht="33.75">
@@ -60317,52 +60366,52 @@
     </row>
     <row r="252" spans="1:1" ht="16.5">
       <c r="A252" s="2" t="s">
-        <v>2044</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="253" spans="1:1" ht="16.5">
       <c r="A253" s="2" t="s">
-        <v>2045</v>
+        <v>2051</v>
       </c>
     </row>
     <row r="254" spans="1:1" ht="16.5">
       <c r="A254" s="2" t="s">
-        <v>2046</v>
+        <v>2052</v>
       </c>
     </row>
     <row r="255" spans="1:1" ht="16.5">
       <c r="A255" s="2" t="s">
-        <v>2047</v>
+        <v>2053</v>
       </c>
     </row>
     <row r="256" spans="1:1" ht="16.5">
       <c r="A256" s="2" t="s">
-        <v>2048</v>
+        <v>2054</v>
       </c>
     </row>
     <row r="257" spans="1:1" ht="33.75">
       <c r="A257" s="2" t="s">
-        <v>2049</v>
+        <v>2055</v>
       </c>
     </row>
     <row r="258" spans="1:1" ht="16.5">
       <c r="A258" s="2" t="s">
-        <v>2050</v>
+        <v>2056</v>
       </c>
     </row>
     <row r="259" spans="1:1" ht="33.75">
       <c r="A259" s="2" t="s">
-        <v>2051</v>
+        <v>2057</v>
       </c>
     </row>
     <row r="260" spans="1:1" ht="16.5">
       <c r="A260" s="2" t="s">
-        <v>2052</v>
+        <v>2058</v>
       </c>
     </row>
     <row r="261" spans="1:1" ht="16.5">
       <c r="A261" s="2" t="s">
-        <v>2053</v>
+        <v>2059</v>
       </c>
     </row>
     <row r="262" spans="1:1" ht="16.5">
@@ -60372,27 +60421,27 @@
     </row>
     <row r="263" spans="1:1" ht="16.5">
       <c r="A263" s="2" t="s">
-        <v>2054</v>
+        <v>2060</v>
       </c>
     </row>
     <row r="264" spans="1:1" ht="33.75">
       <c r="A264" s="2" t="s">
-        <v>2055</v>
+        <v>2061</v>
       </c>
     </row>
     <row r="265" spans="1:1" ht="33.75">
       <c r="A265" s="2" t="s">
-        <v>2056</v>
+        <v>2062</v>
       </c>
     </row>
     <row r="266" spans="1:1" ht="33.75">
       <c r="A266" s="2" t="s">
-        <v>2057</v>
+        <v>2063</v>
       </c>
     </row>
     <row r="267" spans="1:1" ht="16.5">
       <c r="A267" s="2" t="s">
-        <v>2058</v>
+        <v>2064</v>
       </c>
     </row>
     <row r="268" spans="1:1" ht="16.5">
@@ -60402,12 +60451,12 @@
     </row>
     <row r="269" spans="1:1" ht="33.75">
       <c r="A269" s="2" t="s">
-        <v>2059</v>
+        <v>2065</v>
       </c>
     </row>
     <row r="270" spans="1:1" ht="16.5">
       <c r="A270" s="2" t="s">
-        <v>2060</v>
+        <v>2066</v>
       </c>
     </row>
     <row r="271" spans="1:1" ht="16.5">
@@ -60417,32 +60466,32 @@
     </row>
     <row r="272" spans="1:1" ht="16.5">
       <c r="A272" s="2" t="s">
-        <v>2061</v>
+        <v>2067</v>
       </c>
     </row>
     <row r="273" spans="1:1" ht="16.5">
       <c r="A273" s="2" t="s">
-        <v>2062</v>
+        <v>2068</v>
       </c>
     </row>
     <row r="274" spans="1:1" ht="16.5">
       <c r="A274" s="2" t="s">
-        <v>2063</v>
+        <v>2069</v>
       </c>
     </row>
     <row r="275" spans="1:1" ht="16.5">
       <c r="A275" s="2" t="s">
-        <v>2064</v>
+        <v>2070</v>
       </c>
     </row>
     <row r="276" spans="1:1" ht="33.75">
       <c r="A276" s="2" t="s">
-        <v>2065</v>
+        <v>2071</v>
       </c>
     </row>
     <row r="277" spans="1:1" ht="16.5">
       <c r="A277" s="2" t="s">
-        <v>2066</v>
+        <v>2072</v>
       </c>
     </row>
     <row r="278" spans="1:1" ht="33.75">
@@ -60452,7 +60501,7 @@
     </row>
     <row r="279" spans="1:1" ht="50.25">
       <c r="A279" s="2" t="s">
-        <v>2067</v>
+        <v>2073</v>
       </c>
     </row>
     <row r="280" spans="1:1" ht="16.5">
@@ -60462,57 +60511,57 @@
     </row>
     <row r="281" spans="1:1" ht="16.5">
       <c r="A281" s="2" t="s">
-        <v>2068</v>
+        <v>2074</v>
       </c>
     </row>
     <row r="282" spans="1:1" ht="16.5">
       <c r="A282" s="2" t="s">
-        <v>2069</v>
+        <v>2075</v>
       </c>
     </row>
     <row r="283" spans="1:1" ht="16.5">
       <c r="A283" s="2" t="s">
-        <v>2070</v>
+        <v>2076</v>
       </c>
     </row>
     <row r="284" spans="1:1" ht="33.75">
       <c r="A284" s="2" t="s">
-        <v>2071</v>
+        <v>2077</v>
       </c>
     </row>
     <row r="285" spans="1:1" ht="16.5">
       <c r="A285" s="2" t="s">
-        <v>2072</v>
+        <v>2078</v>
       </c>
     </row>
     <row r="286" spans="1:1" ht="16.5">
       <c r="A286" s="2" t="s">
-        <v>2073</v>
+        <v>2079</v>
       </c>
     </row>
     <row r="287" spans="1:1" ht="33.75">
       <c r="A287" s="2" t="s">
-        <v>2074</v>
+        <v>2080</v>
       </c>
     </row>
     <row r="288" spans="1:1" ht="16.5">
       <c r="A288" s="2" t="s">
-        <v>2075</v>
+        <v>2081</v>
       </c>
     </row>
     <row r="289" spans="1:1" ht="16.5">
       <c r="A289" s="2" t="s">
-        <v>2076</v>
+        <v>2082</v>
       </c>
     </row>
     <row r="290" spans="1:1" ht="33.75">
       <c r="A290" s="2" t="s">
-        <v>2077</v>
+        <v>2083</v>
       </c>
     </row>
     <row r="291" spans="1:1" ht="33.75">
       <c r="A291" s="2" t="s">
-        <v>2078</v>
+        <v>2084</v>
       </c>
     </row>
     <row r="292" spans="1:1" ht="16.5">
@@ -60527,62 +60576,62 @@
     </row>
     <row r="294" spans="1:1" ht="16.5">
       <c r="A294" s="2" t="s">
-        <v>2079</v>
+        <v>2085</v>
       </c>
     </row>
     <row r="295" spans="1:1" ht="33.75">
       <c r="A295" s="2" t="s">
-        <v>2080</v>
+        <v>2086</v>
       </c>
     </row>
     <row r="296" spans="1:1" ht="16.5">
       <c r="A296" s="2" t="s">
-        <v>2081</v>
+        <v>2087</v>
       </c>
     </row>
     <row r="297" spans="1:1" ht="33.75">
       <c r="A297" s="2" t="s">
-        <v>2082</v>
+        <v>2088</v>
       </c>
     </row>
     <row r="298" spans="1:1" ht="16.5">
       <c r="A298" s="2" t="s">
-        <v>2083</v>
+        <v>2089</v>
       </c>
     </row>
     <row r="299" spans="1:1" ht="16.5">
       <c r="A299" s="2" t="s">
-        <v>2084</v>
+        <v>2090</v>
       </c>
     </row>
     <row r="300" spans="1:1" ht="16.5">
       <c r="A300" s="2" t="s">
-        <v>2085</v>
+        <v>2091</v>
       </c>
     </row>
     <row r="301" spans="1:1" ht="16.5">
       <c r="A301" s="2" t="s">
-        <v>2086</v>
+        <v>2092</v>
       </c>
     </row>
     <row r="302" spans="1:1" ht="33.75">
       <c r="A302" s="2" t="s">
-        <v>2087</v>
+        <v>2093</v>
       </c>
     </row>
     <row r="303" spans="1:1" ht="16.5">
       <c r="A303" s="2" t="s">
-        <v>2030</v>
+        <v>2036</v>
       </c>
     </row>
     <row r="304" spans="1:1" ht="16.5">
       <c r="A304" s="2" t="s">
-        <v>2088</v>
+        <v>2094</v>
       </c>
     </row>
     <row r="305" spans="1:1" ht="16.5">
       <c r="A305" s="2" t="s">
-        <v>1893</v>
+        <v>1899</v>
       </c>
     </row>
     <row r="306" spans="1:1" ht="16.5">
@@ -60592,12 +60641,12 @@
     </row>
     <row r="307" spans="1:1" ht="16.5">
       <c r="A307" s="2" t="s">
-        <v>2089</v>
+        <v>2095</v>
       </c>
     </row>
     <row r="308" spans="1:1" ht="16.5">
       <c r="A308" s="2" t="s">
-        <v>2090</v>
+        <v>2096</v>
       </c>
     </row>
     <row r="309" spans="1:1" ht="16.5">
@@ -60617,7 +60666,7 @@
     </row>
     <row r="312" spans="1:1" ht="33.75">
       <c r="A312" s="2" t="s">
-        <v>2091</v>
+        <v>2097</v>
       </c>
     </row>
     <row r="313" spans="1:1" ht="16.5">
@@ -60627,22 +60676,22 @@
     </row>
     <row r="314" spans="1:1" ht="16.5">
       <c r="A314" s="2" t="s">
-        <v>2092</v>
+        <v>2098</v>
       </c>
     </row>
     <row r="315" spans="1:1" ht="16.5">
       <c r="A315" s="2" t="s">
-        <v>2093</v>
+        <v>2099</v>
       </c>
     </row>
     <row r="316" spans="1:1" ht="33.75">
       <c r="A316" s="2" t="s">
-        <v>2094</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="317" spans="1:1" ht="16.5">
       <c r="A317" s="2" t="s">
-        <v>2095</v>
+        <v>2101</v>
       </c>
     </row>
     <row r="318" spans="1:1" ht="33.75">
@@ -60657,17 +60706,17 @@
     </row>
     <row r="320" spans="1:1" ht="50.25">
       <c r="A320" s="2" t="s">
-        <v>2096</v>
+        <v>2102</v>
       </c>
     </row>
     <row r="321" spans="1:1" ht="16.5">
       <c r="A321" s="2" t="s">
-        <v>1977</v>
+        <v>1983</v>
       </c>
     </row>
     <row r="322" spans="1:1" ht="16.5">
       <c r="A322" s="2" t="s">
-        <v>2097</v>
+        <v>2103</v>
       </c>
     </row>
     <row r="323" spans="1:1" ht="16.5">
@@ -60677,12 +60726,12 @@
     </row>
     <row r="324" spans="1:1" ht="16.5">
       <c r="A324" s="2" t="s">
-        <v>2098</v>
+        <v>2104</v>
       </c>
     </row>
     <row r="325" spans="1:1" ht="16.5">
       <c r="A325" s="2" t="s">
-        <v>2099</v>
+        <v>2105</v>
       </c>
     </row>
     <row r="326" spans="1:1" ht="16.5">
@@ -60692,7 +60741,7 @@
     </row>
     <row r="327" spans="1:1" ht="16.5">
       <c r="A327" s="2" t="s">
-        <v>2100</v>
+        <v>2106</v>
       </c>
     </row>
     <row r="328" spans="1:1" ht="16.5">
@@ -60702,32 +60751,32 @@
     </row>
     <row r="329" spans="1:1" ht="16.5">
       <c r="A329" s="2" t="s">
-        <v>2101</v>
+        <v>2107</v>
       </c>
     </row>
     <row r="330" spans="1:1" ht="16.5">
       <c r="A330" s="2" t="s">
-        <v>2102</v>
+        <v>2108</v>
       </c>
     </row>
     <row r="331" spans="1:1" ht="50.25">
       <c r="A331" s="2" t="s">
-        <v>2103</v>
+        <v>2109</v>
       </c>
     </row>
     <row r="332" spans="1:1" ht="33.75">
       <c r="A332" s="2" t="s">
-        <v>2104</v>
+        <v>2110</v>
       </c>
     </row>
     <row r="333" spans="1:1" ht="16.5">
       <c r="A333" s="2" t="s">
-        <v>2105</v>
+        <v>2111</v>
       </c>
     </row>
     <row r="334" spans="1:1" ht="16.5">
       <c r="A334" s="2" t="s">
-        <v>2106</v>
+        <v>2112</v>
       </c>
     </row>
     <row r="335" spans="1:1" ht="16.5">
@@ -60737,37 +60786,37 @@
     </row>
     <row r="336" spans="1:1" ht="16.5">
       <c r="A336" s="2" t="s">
-        <v>2107</v>
+        <v>2113</v>
       </c>
     </row>
     <row r="337" spans="1:1" ht="16.5">
       <c r="A337" s="2" t="s">
-        <v>2108</v>
+        <v>2114</v>
       </c>
     </row>
     <row r="338" spans="1:1" ht="16.5">
       <c r="A338" s="2" t="s">
-        <v>2109</v>
+        <v>2115</v>
       </c>
     </row>
     <row r="339" spans="1:1" ht="33.75">
       <c r="A339" s="2" t="s">
-        <v>2110</v>
+        <v>2116</v>
       </c>
     </row>
     <row r="340" spans="1:1" ht="33.75">
       <c r="A340" s="2" t="s">
-        <v>2111</v>
+        <v>2117</v>
       </c>
     </row>
     <row r="341" spans="1:1" ht="16.5">
       <c r="A341" s="2" t="s">
-        <v>2112</v>
+        <v>2118</v>
       </c>
     </row>
     <row r="342" spans="1:1" ht="33.75">
       <c r="A342" s="2" t="s">
-        <v>2113</v>
+        <v>2119</v>
       </c>
     </row>
     <row r="343" spans="1:1" ht="16.5">
@@ -60777,12 +60826,12 @@
     </row>
     <row r="344" spans="1:1" ht="16.5">
       <c r="A344" s="2" t="s">
-        <v>1948</v>
+        <v>1954</v>
       </c>
     </row>
     <row r="345" spans="1:1" ht="33.75">
       <c r="A345" s="2" t="s">
-        <v>2114</v>
+        <v>2120</v>
       </c>
     </row>
     <row r="346" spans="1:1" ht="16.5">
@@ -60802,17 +60851,17 @@
     </row>
     <row r="349" spans="1:1" ht="16.5">
       <c r="A349" s="2" t="s">
-        <v>2115</v>
+        <v>2121</v>
       </c>
     </row>
     <row r="350" spans="1:1" ht="16.5">
       <c r="A350" s="2" t="s">
-        <v>2116</v>
+        <v>2122</v>
       </c>
     </row>
     <row r="351" spans="1:1" ht="16.5">
       <c r="A351" s="2" t="s">
-        <v>2117</v>
+        <v>2123</v>
       </c>
     </row>
     <row r="352" spans="1:1" ht="16.5">
@@ -60822,27 +60871,27 @@
     </row>
     <row r="353" spans="1:1" ht="16.5">
       <c r="A353" s="2" t="s">
-        <v>2118</v>
+        <v>2124</v>
       </c>
     </row>
     <row r="354" spans="1:1" ht="16.5">
       <c r="A354" s="2" t="s">
-        <v>2119</v>
+        <v>2125</v>
       </c>
     </row>
     <row r="355" spans="1:1" ht="33.75">
       <c r="A355" s="2" t="s">
-        <v>2120</v>
+        <v>2126</v>
       </c>
     </row>
     <row r="356" spans="1:1" ht="33.75">
       <c r="A356" s="2" t="s">
-        <v>2121</v>
+        <v>2127</v>
       </c>
     </row>
     <row r="357" spans="1:1" ht="16.5">
       <c r="A357" s="2" t="s">
-        <v>1915</v>
+        <v>1921</v>
       </c>
     </row>
     <row r="358" spans="1:1" ht="16.5">
@@ -60857,12 +60906,12 @@
     </row>
     <row r="360" spans="1:1" ht="16.5">
       <c r="A360" s="2" t="s">
-        <v>2122</v>
+        <v>2128</v>
       </c>
     </row>
     <row r="361" spans="1:1" ht="16.5">
       <c r="A361" s="2" t="s">
-        <v>2123</v>
+        <v>2129</v>
       </c>
     </row>
     <row r="362" spans="1:1" ht="16.5">
@@ -60872,22 +60921,22 @@
     </row>
     <row r="363" spans="1:1" ht="16.5">
       <c r="A363" s="2" t="s">
-        <v>2124</v>
+        <v>2130</v>
       </c>
     </row>
     <row r="364" spans="1:1" ht="16.5">
       <c r="A364" s="2" t="s">
-        <v>2125</v>
+        <v>2131</v>
       </c>
     </row>
     <row r="365" spans="1:1" ht="16.5">
       <c r="A365" s="2" t="s">
-        <v>2126</v>
+        <v>2132</v>
       </c>
     </row>
     <row r="366" spans="1:1" ht="16.5">
       <c r="A366" s="2" t="s">
-        <v>2127</v>
+        <v>2133</v>
       </c>
     </row>
     <row r="367" spans="1:1" ht="16.5">
@@ -60897,57 +60946,57 @@
     </row>
     <row r="368" spans="1:1" ht="16.5">
       <c r="A368" s="2" t="s">
-        <v>2128</v>
+        <v>2134</v>
       </c>
     </row>
     <row r="369" spans="1:1" ht="16.5">
       <c r="A369" s="2" t="s">
-        <v>2129</v>
+        <v>2135</v>
       </c>
     </row>
     <row r="370" spans="1:1" ht="16.5">
       <c r="A370" s="2" t="s">
-        <v>2130</v>
+        <v>2136</v>
       </c>
     </row>
     <row r="371" spans="1:1" ht="16.5">
       <c r="A371" s="2" t="s">
-        <v>2131</v>
+        <v>2137</v>
       </c>
     </row>
     <row r="372" spans="1:1" ht="16.5">
       <c r="A372" s="2" t="s">
-        <v>2132</v>
+        <v>2138</v>
       </c>
     </row>
     <row r="373" spans="1:1" ht="16.5">
       <c r="A373" s="2" t="s">
-        <v>2133</v>
+        <v>2139</v>
       </c>
     </row>
     <row r="374" spans="1:1" ht="16.5">
       <c r="A374" s="2" t="s">
-        <v>2134</v>
+        <v>2140</v>
       </c>
     </row>
     <row r="375" spans="1:1" ht="16.5">
       <c r="A375" s="2" t="s">
-        <v>2135</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="376" spans="1:1" ht="50.25">
       <c r="A376" s="2" t="s">
-        <v>2136</v>
+        <v>2142</v>
       </c>
     </row>
     <row r="377" spans="1:1" ht="16.5">
       <c r="A377" s="2" t="s">
-        <v>2137</v>
+        <v>2143</v>
       </c>
     </row>
     <row r="378" spans="1:1" ht="16.5">
       <c r="A378" s="2" t="s">
-        <v>2138</v>
+        <v>2144</v>
       </c>
     </row>
     <row r="379" spans="1:1" ht="16.5">
@@ -60967,47 +61016,47 @@
     </row>
     <row r="382" spans="1:1" ht="33.75">
       <c r="A382" s="2" t="s">
-        <v>2139</v>
+        <v>2145</v>
       </c>
     </row>
     <row r="383" spans="1:1" ht="16.5">
       <c r="A383" s="2" t="s">
-        <v>2140</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="384" spans="1:1" ht="16.5">
       <c r="A384" s="2" t="s">
-        <v>2141</v>
+        <v>2147</v>
       </c>
     </row>
     <row r="385" spans="1:1" ht="16.5">
       <c r="A385" s="2" t="s">
-        <v>2142</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="386" spans="1:1" ht="16.5">
       <c r="A386" s="2" t="s">
-        <v>2143</v>
+        <v>2149</v>
       </c>
     </row>
     <row r="387" spans="1:1" ht="16.5">
       <c r="A387" s="2" t="s">
-        <v>2144</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="388" spans="1:1" ht="16.5">
       <c r="A388" s="2" t="s">
-        <v>2145</v>
+        <v>2151</v>
       </c>
     </row>
     <row r="389" spans="1:1" ht="16.5">
       <c r="A389" s="2" t="s">
-        <v>2146</v>
+        <v>2152</v>
       </c>
     </row>
     <row r="390" spans="1:1" ht="16.5">
       <c r="A390" s="2" t="s">
-        <v>2147</v>
+        <v>2153</v>
       </c>
     </row>
     <row r="391" spans="1:1" ht="16.5">
@@ -61017,27 +61066,27 @@
     </row>
     <row r="392" spans="1:1" ht="16.5">
       <c r="A392" s="2" t="s">
-        <v>2148</v>
+        <v>2154</v>
       </c>
     </row>
     <row r="393" spans="1:1" ht="16.5">
       <c r="A393" s="2" t="s">
-        <v>2149</v>
+        <v>2155</v>
       </c>
     </row>
     <row r="394" spans="1:1" ht="16.5">
       <c r="A394" s="2" t="s">
-        <v>2150</v>
+        <v>2156</v>
       </c>
     </row>
     <row r="395" spans="1:1" ht="16.5">
       <c r="A395" s="2" t="s">
-        <v>2151</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="396" spans="1:1" ht="16.5">
       <c r="A396" s="2" t="s">
-        <v>2152</v>
+        <v>2158</v>
       </c>
     </row>
     <row r="397" spans="1:1" ht="16.5">
@@ -61057,162 +61106,162 @@
     </row>
     <row r="400" spans="1:1" ht="16.5">
       <c r="A400" s="2" t="s">
-        <v>2153</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="401" spans="1:1" ht="16.5">
       <c r="A401" s="2" t="s">
-        <v>2154</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="402" spans="1:1" ht="16.5">
       <c r="A402" s="2" t="s">
-        <v>2155</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="403" spans="1:1" ht="16.5">
       <c r="A403" s="2" t="s">
-        <v>2156</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="404" spans="1:1" ht="16.5">
       <c r="A404" s="2" t="s">
-        <v>2157</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="405" spans="1:1" ht="33.75">
       <c r="A405" s="2" t="s">
-        <v>2158</v>
+        <v>2164</v>
       </c>
     </row>
     <row r="406" spans="1:1" ht="16.5">
       <c r="A406" s="2" t="s">
-        <v>2159</v>
+        <v>2165</v>
       </c>
     </row>
     <row r="407" spans="1:1" ht="16.5">
       <c r="A407" s="2" t="s">
-        <v>2160</v>
+        <v>2166</v>
       </c>
     </row>
     <row r="408" spans="1:1" ht="33.75">
       <c r="A408" s="2" t="s">
-        <v>2161</v>
+        <v>2167</v>
       </c>
     </row>
     <row r="409" spans="1:1" ht="33.75">
       <c r="A409" s="2" t="s">
-        <v>2162</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="410" spans="1:1" ht="16.5">
       <c r="A410" s="2" t="s">
-        <v>2163</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="411" spans="1:1" ht="16.5">
       <c r="A411" s="2" t="s">
-        <v>2164</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="412" spans="1:1" ht="33.75">
       <c r="A412" s="2" t="s">
-        <v>2165</v>
+        <v>2171</v>
       </c>
     </row>
     <row r="413" spans="1:1" ht="33.75">
       <c r="A413" s="2" t="s">
-        <v>2166</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="414" spans="1:1" ht="16.5">
       <c r="A414" s="2" t="s">
-        <v>2167</v>
+        <v>2173</v>
       </c>
     </row>
     <row r="415" spans="1:1" ht="33.75">
       <c r="A415" s="2" t="s">
-        <v>2168</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="416" spans="1:1" ht="16.5">
       <c r="A416" s="2" t="s">
-        <v>2169</v>
+        <v>2175</v>
       </c>
     </row>
     <row r="417" spans="1:1" ht="16.5">
       <c r="A417" s="2" t="s">
-        <v>2170</v>
+        <v>2176</v>
       </c>
     </row>
     <row r="418" spans="1:1" ht="100.5">
       <c r="A418" s="2" t="s">
-        <v>2171</v>
+        <v>2177</v>
       </c>
     </row>
     <row r="419" spans="1:1" ht="33.75">
       <c r="A419" s="2" t="s">
-        <v>2172</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="420" spans="1:1" ht="16.5">
       <c r="A420" s="2" t="s">
-        <v>2173</v>
+        <v>2179</v>
       </c>
     </row>
     <row r="421" spans="1:1" ht="33.75">
       <c r="A421" s="2" t="s">
-        <v>2174</v>
+        <v>2180</v>
       </c>
     </row>
     <row r="422" spans="1:1" ht="33.75">
       <c r="A422" s="2" t="s">
-        <v>2175</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="423" spans="1:1" ht="33.75">
       <c r="A423" s="2" t="s">
-        <v>2176</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="424" spans="1:1" ht="16.5">
       <c r="A424" s="2" t="s">
-        <v>2177</v>
+        <v>2183</v>
       </c>
     </row>
     <row r="425" spans="1:1" ht="16.5">
       <c r="A425" s="2" t="s">
-        <v>2178</v>
+        <v>2184</v>
       </c>
     </row>
     <row r="426" spans="1:1" ht="33.75">
       <c r="A426" s="2" t="s">
-        <v>2179</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="427" spans="1:1" ht="16.5">
       <c r="A427" s="2" t="s">
-        <v>2180</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="428" spans="1:1" ht="33.75">
       <c r="A428" s="2" t="s">
-        <v>2181</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="429" spans="1:1" ht="16.5">
       <c r="A429" s="2" t="s">
-        <v>1985</v>
+        <v>1991</v>
       </c>
     </row>
     <row r="430" spans="1:1" ht="16.5">
       <c r="A430" s="2" t="s">
-        <v>2182</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="431" spans="1:1" ht="16.5">
       <c r="A431" s="2" t="s">
-        <v>2183</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="432" spans="1:1" ht="16.5">
@@ -61222,12 +61271,12 @@
     </row>
     <row r="433" spans="1:1" ht="33.75">
       <c r="A433" s="2" t="s">
-        <v>2184</v>
+        <v>2190</v>
       </c>
     </row>
     <row r="434" spans="1:1" ht="16.5">
       <c r="A434" s="2" t="s">
-        <v>2185</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="435" spans="1:1" ht="33.75">
@@ -61242,52 +61291,52 @@
     </row>
     <row r="437" spans="1:1" ht="16.5">
       <c r="A437" s="2" t="s">
-        <v>2186</v>
+        <v>2192</v>
       </c>
     </row>
     <row r="438" spans="1:1" ht="16.5">
       <c r="A438" s="2" t="s">
-        <v>2187</v>
+        <v>2193</v>
       </c>
     </row>
     <row r="439" spans="1:1" ht="16.5">
       <c r="A439" s="2" t="s">
-        <v>2188</v>
+        <v>2194</v>
       </c>
     </row>
     <row r="440" spans="1:1" ht="16.5">
       <c r="A440" s="2" t="s">
-        <v>2187</v>
+        <v>2193</v>
       </c>
     </row>
     <row r="441" spans="1:1" ht="16.5">
       <c r="A441" s="2" t="s">
-        <v>2189</v>
+        <v>2195</v>
       </c>
     </row>
     <row r="442" spans="1:1" ht="33.75">
       <c r="A442" s="2" t="s">
-        <v>2190</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="443" spans="1:1" ht="16.5">
       <c r="A443" s="2" t="s">
-        <v>2191</v>
+        <v>2197</v>
       </c>
     </row>
     <row r="444" spans="1:1" ht="16.5">
       <c r="A444" s="2" t="s">
-        <v>2192</v>
+        <v>2198</v>
       </c>
     </row>
     <row r="445" spans="1:1" ht="50.25">
       <c r="A445" s="2" t="s">
-        <v>2193</v>
+        <v>2199</v>
       </c>
     </row>
     <row r="446" spans="1:1" ht="16.5">
       <c r="A446" s="2" t="s">
-        <v>2044</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="447" spans="1:1" ht="16.5">
@@ -61297,62 +61346,62 @@
     </row>
     <row r="448" spans="1:1" ht="16.5">
       <c r="A448" s="2" t="s">
-        <v>2194</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="449" spans="1:1" ht="16.5">
       <c r="A449" s="2" t="s">
-        <v>2195</v>
+        <v>2201</v>
       </c>
     </row>
     <row r="450" spans="1:1" ht="16.5">
       <c r="A450" s="2" t="s">
-        <v>2196</v>
+        <v>2202</v>
       </c>
     </row>
     <row r="451" spans="1:1" ht="33.75">
       <c r="A451" s="2" t="s">
-        <v>2197</v>
+        <v>2203</v>
       </c>
     </row>
     <row r="452" spans="1:1" ht="16.5">
       <c r="A452" s="2" t="s">
-        <v>2198</v>
+        <v>2204</v>
       </c>
     </row>
     <row r="453" spans="1:1" ht="16.5">
       <c r="A453" s="2" t="s">
-        <v>2199</v>
+        <v>2205</v>
       </c>
     </row>
     <row r="454" spans="1:1" ht="16.5">
       <c r="A454" s="2" t="s">
-        <v>2200</v>
+        <v>2206</v>
       </c>
     </row>
     <row r="455" spans="1:1" ht="16.5">
       <c r="A455" s="2" t="s">
-        <v>2201</v>
+        <v>2207</v>
       </c>
     </row>
     <row r="456" spans="1:1" ht="33.75">
       <c r="A456" s="2" t="s">
-        <v>2202</v>
+        <v>2208</v>
       </c>
     </row>
     <row r="457" spans="1:1" ht="16.5">
       <c r="A457" s="2" t="s">
-        <v>2203</v>
+        <v>2209</v>
       </c>
     </row>
     <row r="458" spans="1:1" ht="16.5">
       <c r="A458" s="2" t="s">
-        <v>2204</v>
+        <v>2210</v>
       </c>
     </row>
     <row r="459" spans="1:1" ht="33.75">
       <c r="A459" s="2" t="s">
-        <v>2205</v>
+        <v>2211</v>
       </c>
     </row>
     <row r="460" spans="1:1" ht="16.5">
@@ -61362,32 +61411,32 @@
     </row>
     <row r="461" spans="1:1" ht="16.5">
       <c r="A461" s="2" t="s">
-        <v>2206</v>
+        <v>2212</v>
       </c>
     </row>
     <row r="462" spans="1:1" ht="16.5">
       <c r="A462" s="2" t="s">
-        <v>2207</v>
+        <v>2213</v>
       </c>
     </row>
     <row r="463" spans="1:1" ht="16.5">
       <c r="A463" s="2" t="s">
-        <v>2208</v>
+        <v>2214</v>
       </c>
     </row>
     <row r="464" spans="1:1" ht="33.75">
       <c r="A464" s="2" t="s">
-        <v>2209</v>
+        <v>2215</v>
       </c>
     </row>
     <row r="465" spans="1:1" ht="16.5">
       <c r="A465" s="2" t="s">
-        <v>2210</v>
+        <v>2216</v>
       </c>
     </row>
     <row r="466" spans="1:1" ht="16.5">
       <c r="A466" s="2" t="s">
-        <v>2211</v>
+        <v>2217</v>
       </c>
     </row>
     <row r="467" spans="1:1" ht="33.75">
@@ -61397,237 +61446,237 @@
     </row>
     <row r="468" spans="1:1" ht="16.5">
       <c r="A468" s="2" t="s">
-        <v>2212</v>
+        <v>2218</v>
       </c>
     </row>
     <row r="469" spans="1:1" ht="33.75">
       <c r="A469" s="2" t="s">
-        <v>2213</v>
+        <v>2219</v>
       </c>
     </row>
     <row r="470" spans="1:1" ht="16.5">
       <c r="A470" s="2" t="s">
-        <v>2214</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="471" spans="1:1" ht="16.5">
       <c r="A471" s="2" t="s">
-        <v>2215</v>
+        <v>2221</v>
       </c>
     </row>
     <row r="472" spans="1:1" ht="16.5">
       <c r="A472" s="2" t="s">
-        <v>2216</v>
+        <v>2222</v>
       </c>
     </row>
     <row r="473" spans="1:1" ht="33.75">
       <c r="A473" s="2" t="s">
-        <v>2217</v>
+        <v>2223</v>
       </c>
     </row>
     <row r="474" spans="1:1" ht="33.75">
       <c r="A474" s="2" t="s">
-        <v>2218</v>
+        <v>2224</v>
       </c>
     </row>
     <row r="475" spans="1:1" ht="33.75">
       <c r="A475" s="2" t="s">
-        <v>2219</v>
+        <v>2225</v>
       </c>
     </row>
     <row r="476" spans="1:1" ht="16.5">
       <c r="A476" s="2" t="s">
-        <v>2220</v>
+        <v>2226</v>
       </c>
     </row>
     <row r="477" spans="1:1" ht="16.5">
       <c r="A477" s="2" t="s">
-        <v>2221</v>
+        <v>2227</v>
       </c>
     </row>
     <row r="478" spans="1:1" ht="33.75">
       <c r="A478" s="2" t="s">
-        <v>2222</v>
+        <v>2228</v>
       </c>
     </row>
     <row r="479" spans="1:1" ht="16.5">
       <c r="A479" s="2" t="s">
-        <v>2223</v>
+        <v>2229</v>
       </c>
     </row>
     <row r="480" spans="1:1" ht="16.5">
       <c r="A480" s="2" t="s">
-        <v>2224</v>
+        <v>2230</v>
       </c>
     </row>
     <row r="481" spans="1:1" ht="33.75">
       <c r="A481" s="2" t="s">
-        <v>2225</v>
+        <v>2231</v>
       </c>
     </row>
     <row r="482" spans="1:1" ht="16.5">
       <c r="A482" s="2" t="s">
-        <v>2226</v>
+        <v>2232</v>
       </c>
     </row>
     <row r="483" spans="1:1" ht="16.5">
       <c r="A483" s="2" t="s">
-        <v>2227</v>
+        <v>2233</v>
       </c>
     </row>
     <row r="484" spans="1:1" ht="33.75">
       <c r="A484" s="2" t="s">
-        <v>2228</v>
+        <v>2234</v>
       </c>
     </row>
     <row r="485" spans="1:1" ht="16.5">
       <c r="A485" s="2" t="s">
-        <v>2229</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="486" spans="1:1" ht="16.5">
       <c r="A486" s="2" t="s">
-        <v>2230</v>
+        <v>2236</v>
       </c>
     </row>
     <row r="487" spans="1:1" ht="16.5">
       <c r="A487" s="2" t="s">
-        <v>2231</v>
+        <v>2237</v>
       </c>
     </row>
     <row r="488" spans="1:1" ht="16.5">
       <c r="A488" s="2" t="s">
-        <v>2232</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="489" spans="1:1" ht="16.5">
       <c r="A489" s="2" t="s">
-        <v>2233</v>
+        <v>2239</v>
       </c>
     </row>
     <row r="490" spans="1:1" ht="33.75">
       <c r="A490" s="2" t="s">
-        <v>2234</v>
+        <v>2240</v>
       </c>
     </row>
     <row r="491" spans="1:1" ht="33.75">
       <c r="A491" s="2" t="s">
-        <v>2235</v>
+        <v>2241</v>
       </c>
     </row>
     <row r="492" spans="1:1" ht="16.5">
       <c r="A492" s="2" t="s">
-        <v>2236</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="493" spans="1:1" ht="16.5">
       <c r="A493" s="2" t="s">
-        <v>2237</v>
+        <v>2243</v>
       </c>
     </row>
     <row r="494" spans="1:1" ht="33.75">
       <c r="A494" s="2" t="s">
-        <v>2238</v>
+        <v>2244</v>
       </c>
     </row>
     <row r="495" spans="1:1" ht="33.75">
       <c r="A495" s="2" t="s">
-        <v>2239</v>
+        <v>2245</v>
       </c>
     </row>
     <row r="496" spans="1:1" ht="33.75">
       <c r="A496" s="2" t="s">
-        <v>2240</v>
+        <v>2246</v>
       </c>
     </row>
     <row r="497" spans="1:1" ht="33.75">
       <c r="A497" s="2" t="s">
-        <v>2241</v>
+        <v>2247</v>
       </c>
     </row>
     <row r="498" spans="1:1" ht="16.5">
       <c r="A498" s="2" t="s">
-        <v>2242</v>
+        <v>2248</v>
       </c>
     </row>
     <row r="499" spans="1:1" ht="33.75">
       <c r="A499" s="2" t="s">
-        <v>2243</v>
+        <v>2249</v>
       </c>
     </row>
     <row r="500" spans="1:1" ht="16.5">
       <c r="A500" s="2" t="s">
-        <v>2244</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="501" spans="1:1" ht="16.5">
       <c r="A501" s="2" t="s">
-        <v>2245</v>
+        <v>2251</v>
       </c>
     </row>
     <row r="502" spans="1:1" ht="16.5">
       <c r="A502" s="2" t="s">
-        <v>2246</v>
+        <v>2252</v>
       </c>
     </row>
     <row r="503" spans="1:1" ht="16.5">
       <c r="A503" s="2" t="s">
-        <v>2247</v>
+        <v>2253</v>
       </c>
     </row>
     <row r="504" spans="1:1" ht="16.5">
       <c r="A504" s="2" t="s">
-        <v>2248</v>
+        <v>2254</v>
       </c>
     </row>
     <row r="505" spans="1:1" ht="16.5">
       <c r="A505" s="2" t="s">
-        <v>2249</v>
+        <v>2255</v>
       </c>
     </row>
     <row r="506" spans="1:1" ht="16.5">
       <c r="A506" s="2" t="s">
-        <v>2250</v>
+        <v>2256</v>
       </c>
     </row>
     <row r="507" spans="1:1" ht="33.75">
       <c r="A507" s="2" t="s">
-        <v>2251</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="508" spans="1:1" ht="33.75">
       <c r="A508" s="2" t="s">
-        <v>2252</v>
+        <v>2258</v>
       </c>
     </row>
     <row r="509" spans="1:1" ht="33.75">
       <c r="A509" s="2" t="s">
-        <v>2253</v>
+        <v>2259</v>
       </c>
     </row>
     <row r="510" spans="1:1" ht="16.5">
       <c r="A510" s="2" t="s">
-        <v>2254</v>
+        <v>2260</v>
       </c>
     </row>
     <row r="511" spans="1:1" ht="16.5">
       <c r="A511" s="2" t="s">
-        <v>2255</v>
+        <v>2261</v>
       </c>
     </row>
     <row r="512" spans="1:1" ht="16.5">
       <c r="A512" s="2" t="s">
-        <v>2256</v>
+        <v>2262</v>
       </c>
     </row>
     <row r="513" spans="1:1" ht="16.5">
       <c r="A513" s="2" t="s">
-        <v>2257</v>
+        <v>2263</v>
       </c>
     </row>
     <row r="514" spans="1:1" ht="16.5">
       <c r="A514" s="2" t="s">
-        <v>2258</v>
+        <v>2264</v>
       </c>
     </row>
     <row r="515" spans="1:1" ht="16.5">
@@ -61647,7 +61696,7 @@
     </row>
     <row r="518" spans="1:1" ht="16.5">
       <c r="A518" s="2" t="s">
-        <v>2259</v>
+        <v>2265</v>
       </c>
     </row>
     <row r="519" spans="1:1" ht="16.5">

</xml_diff>